<commit_message>
The Task DELIVERABLES CHECKLIST — ALL 23 OUTPUTS Is Completed
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="cashflow_intelligence" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N94"/>
+  <dimension ref="A1:N95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4187,28 +4187,28 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SHREECEM</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>1.93133294864397</v>
+        <v>0.2905144975221928</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Accrual Risk</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>7.160892839107161</v>
+        <v>0.7401650252861326</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Asset Light</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="n">
-        <v>111.3098672821696</v>
+        <v>24.3832341762802</v>
       </c>
       <c r="H79" t="b">
         <v>0</v>
@@ -4222,80 +4222,80 @@
         </is>
       </c>
       <c r="K79" t="n">
-        <v>3347</v>
+        <v>21632</v>
       </c>
       <c r="L79" t="n">
-        <v>-1710</v>
+        <v>-9896</v>
       </c>
       <c r="M79" t="n">
-        <v>1733</v>
+        <v>74461</v>
       </c>
       <c r="N79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>SHREECEM</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>-3.289718637613709</v>
+        <v>1.93133294864397</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Accrual Risk</t>
+          <t>High Quality</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>0.6472004816375677</v>
+        <v>7.160892839107161</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Asset Light</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="n">
-        <v>-331.7008673577322</v>
+        <v>111.3098672821696</v>
       </c>
       <c r="H80" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I80" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>Growth Funded by Debt</t>
+          <t>Reinvestor</t>
         </is>
       </c>
       <c r="K80" t="n">
-        <v>-31101</v>
+        <v>3347</v>
       </c>
       <c r="L80" t="n">
-        <v>27609</v>
+        <v>-1710</v>
       </c>
       <c r="M80" t="n">
-        <v>9454</v>
+        <v>1733</v>
       </c>
       <c r="N80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SIEMENS</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>0.6144223693892568</v>
+        <v>-3.289718637613709</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Accrual Risk</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>2.257194244604317</v>
+        <v>0.6472004816375677</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -4304,46 +4304,46 @@
       </c>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="n">
-        <v>42.97277409860191</v>
+        <v>-331.7008673577322</v>
       </c>
       <c r="H81" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I81" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
       <c r="K81" t="n">
-        <v>1670</v>
+        <v>-31101</v>
       </c>
       <c r="L81" t="n">
-        <v>-523</v>
+        <v>27609</v>
       </c>
       <c r="M81" t="n">
-        <v>2718</v>
+        <v>9454</v>
       </c>
       <c r="N81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>SIEMENS</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>1.091571467122425</v>
+        <v>0.6144223693892568</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>1.516657390474676</v>
+        <v>2.257194244604317</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -4352,7 +4352,7 @@
       </c>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="n">
-        <v>102.293784294324</v>
+        <v>42.97277409860191</v>
       </c>
       <c r="H82" t="b">
         <v>0</v>
@@ -4366,24 +4366,24 @@
         </is>
       </c>
       <c r="K82" t="n">
-        <v>12135</v>
+        <v>1670</v>
       </c>
       <c r="L82" t="n">
-        <v>-6710</v>
+        <v>-523</v>
       </c>
       <c r="M82" t="n">
-        <v>11117</v>
+        <v>2718</v>
       </c>
       <c r="N82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>1.655555555555555</v>
+        <v>1.091571467122425</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -4391,47 +4391,47 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>11.72608455543965</v>
+        <v>1.516657390474676</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Asset Light</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="n">
-        <v>2.222222222222222</v>
+        <v>102.293784294324</v>
       </c>
       <c r="H83" t="b">
         <v>0</v>
       </c>
       <c r="I83" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>Reinvestor</t>
         </is>
       </c>
       <c r="K83" t="n">
-        <v>1937</v>
+        <v>12135</v>
       </c>
       <c r="L83" t="n">
-        <v>256</v>
+        <v>-6710</v>
       </c>
       <c r="M83" t="n">
-        <v>1170</v>
+        <v>11117</v>
       </c>
       <c r="N83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>TATAMOTORS</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>2.008368819493731</v>
+        <v>1.655555555555555</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -4439,47 +4439,47 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>5.177009550948618</v>
+        <v>11.72608455543965</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="n">
-        <v>133.4664064348237</v>
+        <v>2.222222222222222</v>
       </c>
       <c r="H84" t="b">
         <v>0</v>
       </c>
       <c r="I84" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="K84" t="n">
-        <v>67915</v>
+        <v>1937</v>
       </c>
       <c r="L84" t="n">
-        <v>-37006</v>
+        <v>256</v>
       </c>
       <c r="M84" t="n">
-        <v>33816</v>
+        <v>1170</v>
       </c>
       <c r="N84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>TATAPOWER</t>
+          <t>TATAMOTORS</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>2.860776743129684</v>
+        <v>2.008368819493731</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -4487,16 +4487,16 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>14.21821102868213</v>
+        <v>5.177009550948618</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="n">
-        <v>81.05836929366342</v>
+        <v>133.4664064348237</v>
       </c>
       <c r="H85" t="b">
         <v>0</v>
@@ -4510,24 +4510,24 @@
         </is>
       </c>
       <c r="K85" t="n">
-        <v>12596</v>
+        <v>67915</v>
       </c>
       <c r="L85" t="n">
-        <v>-4497</v>
+        <v>-37006</v>
       </c>
       <c r="M85" t="n">
-        <v>4403</v>
+        <v>33816</v>
       </c>
       <c r="N85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>TATAPOWER</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>8.033636723387415</v>
+        <v>2.860776743129684</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -4535,16 +4535,16 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>6.44897109659204</v>
+        <v>14.21821102868213</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="n">
-        <v>239.3351800554017</v>
+        <v>81.05836929366342</v>
       </c>
       <c r="H86" t="b">
         <v>0</v>
@@ -4558,41 +4558,41 @@
         </is>
       </c>
       <c r="K86" t="n">
-        <v>20301</v>
+        <v>12596</v>
       </c>
       <c r="L86" t="n">
-        <v>-11097</v>
+        <v>-4497</v>
       </c>
       <c r="M86" t="n">
-        <v>2527</v>
+        <v>4403</v>
       </c>
       <c r="N86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>0.9047463575888667</v>
+        <v>8.033636723387415</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
+          <t>High Quality</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>6.44897109659204</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
           <t>Moderate</t>
-        </is>
-      </c>
-      <c r="D87" t="n">
-        <v>2.416277243119302</v>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>Asset Light</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="n">
-        <v>102.9037260743582</v>
+        <v>239.3351800554017</v>
       </c>
       <c r="H87" t="b">
         <v>0</v>
@@ -4602,36 +4602,36 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>Liquidating Assets</t>
+          <t>Reinvestor</t>
         </is>
       </c>
       <c r="K87" t="n">
-        <v>44338</v>
+        <v>20301</v>
       </c>
       <c r="L87" t="n">
-        <v>-48536</v>
+        <v>-11097</v>
       </c>
       <c r="M87" t="n">
-        <v>49006</v>
+        <v>2527</v>
       </c>
       <c r="N87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>1.689006622516556</v>
+        <v>0.9047463575888667</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>2.511624361612928</v>
+        <v>2.416277243119302</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -4640,7 +4640,7 @@
       </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="n">
-        <v>133.9867549668874</v>
+        <v>102.9037260743582</v>
       </c>
       <c r="H88" t="b">
         <v>0</v>
@@ -4650,36 +4650,36 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
+          <t>Liquidating Assets</t>
         </is>
       </c>
       <c r="K88" t="n">
-        <v>6376</v>
+        <v>44338</v>
       </c>
       <c r="L88" t="n">
-        <v>-4767</v>
+        <v>-48536</v>
       </c>
       <c r="M88" t="n">
-        <v>3775</v>
+        <v>49006</v>
       </c>
       <c r="N88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>0.5226641998149861</v>
+        <v>1.689006622516556</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>High Quality</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>0.3470564471702964</v>
+        <v>2.511624361612928</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -4688,7 +4688,7 @@
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="n">
-        <v>46.43848288621646</v>
+        <v>133.9867549668874</v>
       </c>
       <c r="H89" t="b">
         <v>0</v>
@@ -4702,32 +4702,32 @@
         </is>
       </c>
       <c r="K89" t="n">
-        <v>1695</v>
+        <v>6376</v>
       </c>
       <c r="L89" t="n">
-        <v>-1329</v>
+        <v>-4767</v>
       </c>
       <c r="M89" t="n">
-        <v>3243</v>
+        <v>3775</v>
       </c>
       <c r="N89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>TORNTPHARM</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>1.754027926960258</v>
+        <v>0.5226641998149861</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>1.415678640948505</v>
+        <v>0.3470564471702964</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -4736,7 +4736,7 @@
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="n">
-        <v>166.8098818474758</v>
+        <v>46.43848288621646</v>
       </c>
       <c r="H90" t="b">
         <v>0</v>
@@ -4750,41 +4750,41 @@
         </is>
       </c>
       <c r="K90" t="n">
-        <v>3266</v>
+        <v>1695</v>
       </c>
       <c r="L90" t="n">
-        <v>-2780</v>
+        <v>-1329</v>
       </c>
       <c r="M90" t="n">
-        <v>1862</v>
+        <v>3243</v>
       </c>
       <c r="N90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>TORNTPHARM</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>0.7457158651188502</v>
+        <v>1.754027926960258</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>High Quality</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>3.381031613976705</v>
+        <v>1.415678640948505</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Asset Light</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="n">
-        <v>46.489773355445</v>
+        <v>166.8098818474758</v>
       </c>
       <c r="H91" t="b">
         <v>0</v>
@@ -4798,120 +4798,120 @@
         </is>
       </c>
       <c r="K91" t="n">
-        <v>1349</v>
+        <v>3266</v>
       </c>
       <c r="L91" t="n">
-        <v>-629</v>
+        <v>-2780</v>
       </c>
       <c r="M91" t="n">
-        <v>1809</v>
+        <v>1862</v>
       </c>
       <c r="N91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>TVSMOTOR</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>-0.5983763132760267</v>
+        <v>0.7457158651188502</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Accrual Risk</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>2.334095042671268</v>
+        <v>3.381031613976705</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Asset Light</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="n">
-        <v>-107.6408787010506</v>
+        <v>46.489773355445</v>
       </c>
       <c r="H92" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I92" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>Growth Funded by Debt</t>
+          <t>Reinvestor</t>
         </is>
       </c>
       <c r="K92" t="n">
-        <v>-1253</v>
+        <v>1349</v>
       </c>
       <c r="L92" t="n">
-        <v>2759</v>
+        <v>-629</v>
       </c>
       <c r="M92" t="n">
-        <v>2094</v>
+        <v>1809</v>
       </c>
       <c r="N92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>TVSMOTOR</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>1.743122200895713</v>
+        <v>-0.5983763132760267</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Accrual Risk</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>12.32384985347112</v>
+        <v>2.334095042671268</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Asset Light</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="n">
-        <v>33.73320537428023</v>
+        <v>-107.6408787010506</v>
       </c>
       <c r="H93" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I93" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
       <c r="K93" t="n">
-        <v>10898</v>
+        <v>-1253</v>
       </c>
       <c r="L93" t="n">
-        <v>-1926</v>
+        <v>2759</v>
       </c>
       <c r="M93" t="n">
-        <v>6252</v>
+        <v>2094</v>
       </c>
       <c r="N93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>UNIONBANK</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>1.219407733724914</v>
+        <v>1.743122200895713</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -4919,38 +4919,86 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>1.302097928225822</v>
+        <v>12.32384985347112</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Asset Light</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="n">
+        <v>33.73320537428023</v>
+      </c>
+      <c r="H94" t="b">
+        <v>0</v>
+      </c>
+      <c r="I94" t="b">
+        <v>1</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="K94" t="n">
+        <v>10898</v>
+      </c>
+      <c r="L94" t="n">
+        <v>-1926</v>
+      </c>
+      <c r="M94" t="n">
+        <v>6252</v>
+      </c>
+      <c r="N94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>UNIONBANK</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>1.219407733724914</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>High Quality</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>1.302097928225822</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Asset Light</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="n">
         <v>113.4116495349976</v>
       </c>
-      <c r="H94" t="b">
-        <v>0</v>
-      </c>
-      <c r="I94" t="b">
-        <v>1</v>
-      </c>
-      <c r="J94" t="inlineStr">
-        <is>
-          <t>Reinvestor</t>
-        </is>
-      </c>
-      <c r="K94" t="n">
+      <c r="H95" t="b">
+        <v>0</v>
+      </c>
+      <c r="I95" t="b">
+        <v>1</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="K95" t="n">
         <v>19930</v>
       </c>
-      <c r="L94" t="n">
+      <c r="L95" t="n">
         <v>-11489</v>
       </c>
-      <c r="M94" t="n">
+      <c r="M95" t="n">
         <v>16344</v>
       </c>
-      <c r="N94" t="inlineStr"/>
+      <c r="N95" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>